<commit_message>
Excel: suppress green error-check triangles in all models
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBVdxY5GcRU6xZ4qeSea35
</commit_message>
<xml_diff>
--- a/RAMEN_FINMODEL_INTERNAL_EN_BONUS_COMPENSATION.xlsx
+++ b/RAMEN_FINMODEL_INTERNAL_EN_BONUS_COMPENSATION.xlsx
@@ -3703,6 +3703,9 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:AI59" evalError="1" formula="1" formulaRange="1" unlockedFormula="1" numberStoredAsText="1" emptyCellReference="1" twoDigitTextYear="1" listDataValidation="1" calculatedColumn="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -5864,6 +5867,9 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:AI59" evalError="1" formula="1" formulaRange="1" unlockedFormula="1" numberStoredAsText="1" emptyCellReference="1" twoDigitTextYear="1" listDataValidation="1" calculatedColumn="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -6464,6 +6470,9 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:H45" evalError="1" formula="1" formulaRange="1" unlockedFormula="1" numberStoredAsText="1" emptyCellReference="1" twoDigitTextYear="1" listDataValidation="1" calculatedColumn="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -7061,6 +7070,9 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:H44" evalError="1" formula="1" formulaRange="1" unlockedFormula="1" numberStoredAsText="1" emptyCellReference="1" twoDigitTextYear="1" listDataValidation="1" calculatedColumn="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -8044,5 +8056,8 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:N49" evalError="1" formula="1" formulaRange="1" unlockedFormula="1" numberStoredAsText="1" emptyCellReference="1" twoDigitTextYear="1" listDataValidation="1" calculatedColumn="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>